<commit_message>
Modelo posicao-estoque.xlsx: adiciona 8 linhas de dados fictícios
https://claude.ai/code/session_01GB592wHtRegLJEtgwh4ZdP
</commit_message>
<xml_diff>
--- a/painel/assets/modelos/posicao-estoque.xlsx
+++ b/painel/assets/modelos/posicao-estoque.xlsx
@@ -69,9 +69,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF999999"/>
-      <sz val="9"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="9">
@@ -103,12 +101,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
+        <fgColor rgb="FF155724"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF155724"/>
+        <fgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
@@ -143,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -154,21 +152,22 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -536,11 +535,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
@@ -583,69 +582,239 @@
           <t>Responsável pela contagem:</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Nome do Responsável</t>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>João Responsável</t>
         </is>
       </c>
     </row>
     <row r="6" ht="8" customHeight="1"/>
     <row r="7" ht="8" customHeight="1"/>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Tipo / Categoria</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Unidade</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Estoque Encontrado</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>← EXEMPLO (esta linha é ignorada)</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>← LINHA DE EXEMPLO (ignorada pelo importador)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Tubulação</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>75,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>MAT-001</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Tubo PVC 200mm</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Tubulação</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>120,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>MAT-002</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Conexões</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>45,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>MAT-003</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Cimento</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>MAT-004</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Areia</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>12,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>MAT-005</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Brita</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>8,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>MAT-006</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>EPI - Luvas</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>par</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>30,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>MAT-007</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>EPI - Capacete</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>10,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>MAT-008</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Fita veda rosca</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>